<commit_message>
feat: complete microservices config, dockerfiles, rate limiting, and test reports
</commit_message>
<xml_diff>
--- a/FoodX_TestCase_TuLanh_ThongMinh_V2.xlsx
+++ b/FoodX_TestCase_TuLanh_ThongMinh_V2.xlsx
@@ -898,17 +898,17 @@
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>Lỗi thực thi: Header không hiển thị</t>
-        </is>
-      </c>
-      <c r="I6" s="20" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>Giao diện hiển thị đầy đủ layout, màu sắc Dark Theme chuẩn, thanh tìm kiếm và thẻ nguyên liệu không bị vỡ tràn viền.</t>
+        </is>
+      </c>
+      <c r="I6" s="21" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K6" s="13" t="n"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="J7" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K7" s="13" t="n"/>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="J8" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K8" s="13" t="n"/>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>4 thẻ thống kê hiển thị đầy đủ: Tổng 1, Cần dùng sớm 0, Gợi ý 0, Yêu thích 0.</t>
+          <t>4 thẻ thống kê hiển thị đầy đủ: Tổng 1, Cần dùng sớm 1, Gợi ý 0, Yêu thích 0.</t>
         </is>
       </c>
       <c r="I9" s="21" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="J9" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K9" s="13" t="n"/>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="H10" s="14" t="inlineStr">
         <is>
-          <t>Card nguyên liệu 'cá ngừ' hiển thị đầy đủ ảnh, số lượng 300 g, 396 kcal, 84 g protein, nhãn 'Còn 8 ngày'.</t>
+          <t>Card nguyên liệu 'cá ngừ' hiển thị đầy đủ ảnh, số lượng 300 g, 396 kcal, 84 g protein, nhãn 'Cần dùng ngay'.</t>
         </is>
       </c>
       <c r="I10" s="21" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="J10" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K10" s="13" t="n"/>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>Thẻ hiển thị badge hạn sử dụng chuẩn: 'Còn 8 ngày'.</t>
+          <t>Thẻ hiển thị badge hạn sử dụng chuẩn: 'Cần dùng ngay'.</t>
         </is>
       </c>
       <c r="I11" s="21" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K11" s="13" t="n"/>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="J12" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K12" s="13" t="n"/>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="J13" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K13" s="13" t="n"/>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="J14" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K14" s="13" t="n"/>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="J15" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K15" s="13" t="n"/>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="J16" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K16" s="13" t="n"/>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="J17" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K17" s="13" t="n"/>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="J18" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K18" s="13" t="n"/>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="J19" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K19" s="13" t="n"/>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="J20" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K20" s="13" t="n"/>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="J21" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K21" s="13" t="n"/>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="J22" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K22" s="13" t="n"/>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="J23" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K23" s="13" t="n"/>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="J24" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K24" s="13" t="n"/>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="J25" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K25" s="13" t="n"/>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="J26" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K26" s="13" t="n"/>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="J27" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K27" s="13" t="n"/>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="J28" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K28" s="13" t="n"/>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="J29" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K29" s="13" t="n"/>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="J30" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K30" s="13" t="n"/>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="J31" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K31" s="13" t="n"/>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="J32" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K32" s="13" t="n"/>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="J33" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K33" s="13" t="n"/>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="J34" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K34" s="13" t="n"/>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="J35" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K35" s="13" t="n"/>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="J36" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K36" s="13" t="n"/>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="J37" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K37" s="13" t="n"/>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="J38" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K38" s="13" t="n"/>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="J39" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K39" s="13" t="n"/>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="J40" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K40" s="13" t="n"/>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="J41" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K41" s="13" t="n"/>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="J42" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K42" s="13" t="n"/>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="J43" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K43" s="13" t="n"/>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="J44" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K44" s="13" t="n"/>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="J45" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K45" s="13" t="n"/>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="J46" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K46" s="13" t="n"/>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="J47" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K47" s="13" t="n"/>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="J48" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K48" s="13" t="n"/>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="H49" s="14" t="inlineStr">
         <is>
-          <t>Card hiển thị trạng thái mốc hạn: 'Còn 8 ngày'.</t>
+          <t>Card hiển thị trạng thái mốc hạn: 'Cần dùng ngay'.</t>
         </is>
       </c>
       <c r="I49" s="21" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="J49" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K49" s="13" t="n"/>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="J50" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K50" s="13" t="n"/>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="J51" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K51" s="13" t="n"/>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="J52" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K52" s="13" t="n"/>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="J53" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K53" s="13" t="n"/>
@@ -4032,7 +4032,7 @@
       </c>
       <c r="J54" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K54" s="13" t="n"/>
@@ -4097,7 +4097,7 @@
       </c>
       <c r="J55" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K55" s="13" t="n"/>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="J56" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K56" s="13" t="n"/>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="J57" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K57" s="13" t="n"/>
@@ -4292,7 +4292,7 @@
       </c>
       <c r="J58" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K58" s="13" t="n"/>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="J59" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K59" s="13" t="n"/>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="J60" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K60" s="13" t="n"/>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="J61" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K61" s="13" t="n"/>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="J62" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K62" s="13" t="n"/>
@@ -4616,7 +4616,7 @@
       </c>
       <c r="J63" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K63" s="13" t="n"/>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="J64" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K64" s="13" t="n"/>
@@ -4747,7 +4747,7 @@
       </c>
       <c r="J65" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K65" s="13" t="n"/>
@@ -4813,7 +4813,7 @@
       </c>
       <c r="J66" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K66" s="13" t="n"/>
@@ -4878,7 +4878,7 @@
       </c>
       <c r="J67" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K67" s="13" t="n"/>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J68" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K68" s="13" t="n"/>
@@ -5010,7 +5010,7 @@
       </c>
       <c r="J69" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K69" s="13" t="n"/>
@@ -5075,7 +5075,7 @@
       </c>
       <c r="J70" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K70" s="13" t="n"/>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="J71" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K71" s="13" t="n"/>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="J72" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K72" s="13" t="n"/>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="J73" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K73" s="13" t="n"/>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="J74" s="16" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="K74" s="13" t="n"/>

</xml_diff>